<commit_message>
analysis added, year range extended to 2100, bug with directories fixed
</commit_message>
<xml_diff>
--- a/excel/t1.xlsx
+++ b/excel/t1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/72c13503b0c010a4/Desktop/Прект_10/.venv/excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/72c13503b0c010a4/Desktop/Прект_10/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="11_AD4DF75460589B3ACB728430E75B765A5BDEDD91" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8F8A90F3-60AD-467F-9439-FAC9AC6CCD6E}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="11_AD4DF75460589B3ACB728430E75B765A5BDEDD91" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7D98090-6A3E-40A4-8063-6085E1BE6C65}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6380" yWindow="4030" windowWidth="28800" windowHeight="15910" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -99,7 +99,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -194,11 +194,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -219,6 +230,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -501,7 +515,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
@@ -791,7 +805,7 @@
         <v>380</v>
       </c>
       <c r="D13" s="7">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E13" s="7">
         <v>5</v>
@@ -814,7 +828,7 @@
         <v>390</v>
       </c>
       <c r="D14" s="7">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E14" s="7">
         <v>5</v>
@@ -837,7 +851,7 @@
         <v>400</v>
       </c>
       <c r="D15" s="7">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E15" s="7">
         <v>5</v>
@@ -860,7 +874,7 @@
         <v>410</v>
       </c>
       <c r="D16" s="7">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E16" s="7">
         <v>5</v>
@@ -883,7 +897,7 @@
         <v>420</v>
       </c>
       <c r="D17" s="7">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E17" s="7">
         <v>5</v>
@@ -906,7 +920,7 @@
         <v>430</v>
       </c>
       <c r="D18" s="7">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E18" s="7">
         <v>5</v>
@@ -929,7 +943,7 @@
         <v>440</v>
       </c>
       <c r="D19" s="7">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E19" s="7">
         <v>5</v>
@@ -1007,6 +1021,1156 @@
         <v>6</v>
       </c>
       <c r="G22" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="3">
+        <v>2051</v>
+      </c>
+      <c r="B23" s="7">
+        <v>491</v>
+      </c>
+      <c r="C23" s="7">
+        <v>480</v>
+      </c>
+      <c r="D23" s="7">
+        <v>0</v>
+      </c>
+      <c r="E23" s="7">
+        <v>5</v>
+      </c>
+      <c r="F23" s="7">
+        <v>6</v>
+      </c>
+      <c r="G23" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" s="5">
+        <v>2052</v>
+      </c>
+      <c r="B24" s="7">
+        <v>501</v>
+      </c>
+      <c r="C24" s="7">
+        <v>490</v>
+      </c>
+      <c r="D24" s="7">
+        <v>0</v>
+      </c>
+      <c r="E24" s="7">
+        <v>5</v>
+      </c>
+      <c r="F24" s="7">
+        <v>6</v>
+      </c>
+      <c r="G24" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" s="7">
+        <v>2053</v>
+      </c>
+      <c r="B25" s="7">
+        <v>511</v>
+      </c>
+      <c r="C25" s="7">
+        <v>500</v>
+      </c>
+      <c r="D25" s="7">
+        <v>0</v>
+      </c>
+      <c r="E25" s="7">
+        <v>5</v>
+      </c>
+      <c r="F25" s="7">
+        <v>6</v>
+      </c>
+      <c r="G25" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" s="7">
+        <v>2054</v>
+      </c>
+      <c r="B26" s="7">
+        <v>521</v>
+      </c>
+      <c r="C26" s="7">
+        <v>510</v>
+      </c>
+      <c r="D26" s="7">
+        <v>0</v>
+      </c>
+      <c r="E26" s="7">
+        <v>5</v>
+      </c>
+      <c r="F26" s="7">
+        <v>6</v>
+      </c>
+      <c r="G26" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27" s="7">
+        <v>2055</v>
+      </c>
+      <c r="B27" s="7">
+        <v>531</v>
+      </c>
+      <c r="C27" s="7">
+        <v>520</v>
+      </c>
+      <c r="D27" s="7">
+        <v>0</v>
+      </c>
+      <c r="E27" s="7">
+        <v>5</v>
+      </c>
+      <c r="F27" s="7">
+        <v>6</v>
+      </c>
+      <c r="G27" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A28" s="7">
+        <v>2056</v>
+      </c>
+      <c r="B28" s="7">
+        <v>541</v>
+      </c>
+      <c r="C28" s="7">
+        <v>530</v>
+      </c>
+      <c r="D28" s="7">
+        <v>0</v>
+      </c>
+      <c r="E28" s="7">
+        <v>5</v>
+      </c>
+      <c r="F28" s="7">
+        <v>6</v>
+      </c>
+      <c r="G28" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29" s="7">
+        <v>2057</v>
+      </c>
+      <c r="B29" s="7">
+        <v>551</v>
+      </c>
+      <c r="C29" s="7">
+        <v>540</v>
+      </c>
+      <c r="D29" s="7">
+        <v>0</v>
+      </c>
+      <c r="E29" s="7">
+        <v>5</v>
+      </c>
+      <c r="F29" s="7">
+        <v>6</v>
+      </c>
+      <c r="G29" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30" s="7">
+        <v>2058</v>
+      </c>
+      <c r="B30" s="7">
+        <v>561</v>
+      </c>
+      <c r="C30" s="7">
+        <v>550</v>
+      </c>
+      <c r="D30" s="7">
+        <v>0</v>
+      </c>
+      <c r="E30" s="7">
+        <v>5</v>
+      </c>
+      <c r="F30" s="7">
+        <v>6</v>
+      </c>
+      <c r="G30" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A31" s="7">
+        <v>2059</v>
+      </c>
+      <c r="B31" s="7">
+        <v>571</v>
+      </c>
+      <c r="C31" s="7">
+        <v>560</v>
+      </c>
+      <c r="D31" s="7">
+        <v>0</v>
+      </c>
+      <c r="E31" s="7">
+        <v>5</v>
+      </c>
+      <c r="F31" s="7">
+        <v>6</v>
+      </c>
+      <c r="G31" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A32" s="7">
+        <v>2060</v>
+      </c>
+      <c r="B32" s="7">
+        <v>581</v>
+      </c>
+      <c r="C32" s="7">
+        <v>570</v>
+      </c>
+      <c r="D32" s="7">
+        <v>0</v>
+      </c>
+      <c r="E32" s="7">
+        <v>5</v>
+      </c>
+      <c r="F32" s="7">
+        <v>6</v>
+      </c>
+      <c r="G32" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A33" s="7">
+        <v>2061</v>
+      </c>
+      <c r="B33" s="7">
+        <v>591</v>
+      </c>
+      <c r="C33" s="7">
+        <v>580</v>
+      </c>
+      <c r="D33" s="7">
+        <v>0</v>
+      </c>
+      <c r="E33" s="7">
+        <v>5</v>
+      </c>
+      <c r="F33" s="7">
+        <v>6</v>
+      </c>
+      <c r="G33" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A34" s="7">
+        <v>2062</v>
+      </c>
+      <c r="B34" s="7">
+        <v>601</v>
+      </c>
+      <c r="C34" s="7">
+        <v>590</v>
+      </c>
+      <c r="D34" s="7">
+        <v>0</v>
+      </c>
+      <c r="E34" s="7">
+        <v>5</v>
+      </c>
+      <c r="F34" s="7">
+        <v>6</v>
+      </c>
+      <c r="G34" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A35" s="7">
+        <v>2063</v>
+      </c>
+      <c r="B35" s="7">
+        <v>611</v>
+      </c>
+      <c r="C35" s="7">
+        <v>600</v>
+      </c>
+      <c r="D35" s="7">
+        <v>0</v>
+      </c>
+      <c r="E35" s="7">
+        <v>5</v>
+      </c>
+      <c r="F35" s="7">
+        <v>6</v>
+      </c>
+      <c r="G35" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A36" s="7">
+        <v>2064</v>
+      </c>
+      <c r="B36" s="7">
+        <v>621</v>
+      </c>
+      <c r="C36" s="7">
+        <v>610</v>
+      </c>
+      <c r="D36" s="7">
+        <v>0</v>
+      </c>
+      <c r="E36" s="7">
+        <v>5</v>
+      </c>
+      <c r="F36" s="7">
+        <v>6</v>
+      </c>
+      <c r="G36" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A37" s="7">
+        <v>2065</v>
+      </c>
+      <c r="B37" s="7">
+        <v>631</v>
+      </c>
+      <c r="C37" s="7">
+        <v>620</v>
+      </c>
+      <c r="D37" s="7">
+        <v>0</v>
+      </c>
+      <c r="E37" s="7">
+        <v>5</v>
+      </c>
+      <c r="F37" s="7">
+        <v>6</v>
+      </c>
+      <c r="G37" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A38" s="7">
+        <v>2066</v>
+      </c>
+      <c r="B38" s="7">
+        <v>641</v>
+      </c>
+      <c r="C38" s="7">
+        <v>630</v>
+      </c>
+      <c r="D38" s="7">
+        <v>0</v>
+      </c>
+      <c r="E38" s="7">
+        <v>5</v>
+      </c>
+      <c r="F38" s="7">
+        <v>6</v>
+      </c>
+      <c r="G38" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A39" s="7">
+        <v>2067</v>
+      </c>
+      <c r="B39" s="7">
+        <v>651</v>
+      </c>
+      <c r="C39" s="7">
+        <v>640</v>
+      </c>
+      <c r="D39" s="7">
+        <v>0</v>
+      </c>
+      <c r="E39" s="7">
+        <v>5</v>
+      </c>
+      <c r="F39" s="7">
+        <v>6</v>
+      </c>
+      <c r="G39" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A40" s="3">
+        <v>2068</v>
+      </c>
+      <c r="B40" s="7">
+        <v>661</v>
+      </c>
+      <c r="C40" s="7">
+        <v>650</v>
+      </c>
+      <c r="D40" s="7">
+        <v>0</v>
+      </c>
+      <c r="E40" s="7">
+        <v>5</v>
+      </c>
+      <c r="F40" s="7">
+        <v>6</v>
+      </c>
+      <c r="G40" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A41" s="5">
+        <v>2069</v>
+      </c>
+      <c r="B41" s="7">
+        <v>671</v>
+      </c>
+      <c r="C41" s="7">
+        <v>660</v>
+      </c>
+      <c r="D41" s="7">
+        <v>0</v>
+      </c>
+      <c r="E41" s="7">
+        <v>5</v>
+      </c>
+      <c r="F41" s="7">
+        <v>6</v>
+      </c>
+      <c r="G41" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A42" s="7">
+        <v>2070</v>
+      </c>
+      <c r="B42" s="7">
+        <v>681</v>
+      </c>
+      <c r="C42" s="7">
+        <v>670</v>
+      </c>
+      <c r="D42" s="7">
+        <v>0</v>
+      </c>
+      <c r="E42" s="7">
+        <v>5</v>
+      </c>
+      <c r="F42" s="7">
+        <v>6</v>
+      </c>
+      <c r="G42" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A43" s="7">
+        <v>2071</v>
+      </c>
+      <c r="B43" s="7">
+        <v>691</v>
+      </c>
+      <c r="C43" s="7">
+        <v>680</v>
+      </c>
+      <c r="D43" s="7">
+        <v>0</v>
+      </c>
+      <c r="E43" s="7">
+        <v>5</v>
+      </c>
+      <c r="F43" s="7">
+        <v>6</v>
+      </c>
+      <c r="G43" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A44" s="7">
+        <v>2072</v>
+      </c>
+      <c r="B44" s="7">
+        <v>701</v>
+      </c>
+      <c r="C44" s="7">
+        <v>690</v>
+      </c>
+      <c r="D44" s="7">
+        <v>0</v>
+      </c>
+      <c r="E44" s="7">
+        <v>5</v>
+      </c>
+      <c r="F44" s="7">
+        <v>6</v>
+      </c>
+      <c r="G44" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A45" s="7">
+        <v>2073</v>
+      </c>
+      <c r="B45" s="7">
+        <v>711</v>
+      </c>
+      <c r="C45" s="7">
+        <v>700</v>
+      </c>
+      <c r="D45" s="7">
+        <v>0</v>
+      </c>
+      <c r="E45" s="7">
+        <v>5</v>
+      </c>
+      <c r="F45" s="7">
+        <v>6</v>
+      </c>
+      <c r="G45" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A46" s="7">
+        <v>2074</v>
+      </c>
+      <c r="B46" s="7">
+        <v>721</v>
+      </c>
+      <c r="C46" s="7">
+        <v>710</v>
+      </c>
+      <c r="D46" s="7">
+        <v>0</v>
+      </c>
+      <c r="E46" s="7">
+        <v>5</v>
+      </c>
+      <c r="F46" s="7">
+        <v>6</v>
+      </c>
+      <c r="G46" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A47" s="7">
+        <v>2075</v>
+      </c>
+      <c r="B47" s="7">
+        <v>731</v>
+      </c>
+      <c r="C47" s="7">
+        <v>720</v>
+      </c>
+      <c r="D47" s="7">
+        <v>0</v>
+      </c>
+      <c r="E47" s="7">
+        <v>5</v>
+      </c>
+      <c r="F47" s="7">
+        <v>6</v>
+      </c>
+      <c r="G47" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A48" s="7">
+        <v>2076</v>
+      </c>
+      <c r="B48" s="7">
+        <v>741</v>
+      </c>
+      <c r="C48" s="7">
+        <v>730</v>
+      </c>
+      <c r="D48" s="7">
+        <v>0</v>
+      </c>
+      <c r="E48" s="7">
+        <v>5</v>
+      </c>
+      <c r="F48" s="7">
+        <v>6</v>
+      </c>
+      <c r="G48" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A49" s="7">
+        <v>2077</v>
+      </c>
+      <c r="B49" s="7">
+        <v>751</v>
+      </c>
+      <c r="C49" s="7">
+        <v>740</v>
+      </c>
+      <c r="D49" s="7">
+        <v>0</v>
+      </c>
+      <c r="E49" s="7">
+        <v>5</v>
+      </c>
+      <c r="F49" s="7">
+        <v>6</v>
+      </c>
+      <c r="G49" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A50" s="7">
+        <v>2078</v>
+      </c>
+      <c r="B50" s="7">
+        <v>761</v>
+      </c>
+      <c r="C50" s="7">
+        <v>750</v>
+      </c>
+      <c r="D50" s="7">
+        <v>0</v>
+      </c>
+      <c r="E50" s="7">
+        <v>5</v>
+      </c>
+      <c r="F50" s="7">
+        <v>6</v>
+      </c>
+      <c r="G50" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A51" s="7">
+        <v>2079</v>
+      </c>
+      <c r="B51" s="7">
+        <v>771</v>
+      </c>
+      <c r="C51" s="7">
+        <v>760</v>
+      </c>
+      <c r="D51" s="7">
+        <v>0</v>
+      </c>
+      <c r="E51" s="7">
+        <v>5</v>
+      </c>
+      <c r="F51" s="7">
+        <v>6</v>
+      </c>
+      <c r="G51" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A52" s="7">
+        <v>2080</v>
+      </c>
+      <c r="B52" s="7">
+        <v>781</v>
+      </c>
+      <c r="C52" s="7">
+        <v>770</v>
+      </c>
+      <c r="D52" s="7">
+        <v>0</v>
+      </c>
+      <c r="E52" s="7">
+        <v>5</v>
+      </c>
+      <c r="F52" s="7">
+        <v>6</v>
+      </c>
+      <c r="G52" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A53" s="7">
+        <v>2081</v>
+      </c>
+      <c r="B53" s="7">
+        <v>791</v>
+      </c>
+      <c r="C53" s="7">
+        <v>780</v>
+      </c>
+      <c r="D53" s="7">
+        <v>0</v>
+      </c>
+      <c r="E53" s="7">
+        <v>5</v>
+      </c>
+      <c r="F53" s="7">
+        <v>6</v>
+      </c>
+      <c r="G53" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A54" s="7">
+        <v>2082</v>
+      </c>
+      <c r="B54" s="7">
+        <v>801</v>
+      </c>
+      <c r="C54" s="7">
+        <v>790</v>
+      </c>
+      <c r="D54" s="7">
+        <v>0</v>
+      </c>
+      <c r="E54" s="7">
+        <v>5</v>
+      </c>
+      <c r="F54" s="7">
+        <v>6</v>
+      </c>
+      <c r="G54" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A55" s="7">
+        <v>2083</v>
+      </c>
+      <c r="B55" s="7">
+        <v>811</v>
+      </c>
+      <c r="C55" s="7">
+        <v>800</v>
+      </c>
+      <c r="D55" s="7">
+        <v>0</v>
+      </c>
+      <c r="E55" s="7">
+        <v>5</v>
+      </c>
+      <c r="F55" s="7">
+        <v>6</v>
+      </c>
+      <c r="G55" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A56" s="7">
+        <v>2084</v>
+      </c>
+      <c r="B56" s="7">
+        <v>821</v>
+      </c>
+      <c r="C56" s="7">
+        <v>810</v>
+      </c>
+      <c r="D56" s="7">
+        <v>0</v>
+      </c>
+      <c r="E56" s="7">
+        <v>5</v>
+      </c>
+      <c r="F56" s="7">
+        <v>6</v>
+      </c>
+      <c r="G56" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A57" s="3">
+        <v>2085</v>
+      </c>
+      <c r="B57" s="7">
+        <v>831</v>
+      </c>
+      <c r="C57" s="7">
+        <v>820</v>
+      </c>
+      <c r="D57" s="7">
+        <v>0</v>
+      </c>
+      <c r="E57" s="7">
+        <v>5</v>
+      </c>
+      <c r="F57" s="7">
+        <v>6</v>
+      </c>
+      <c r="G57" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A58" s="5">
+        <v>2086</v>
+      </c>
+      <c r="B58" s="7">
+        <v>841</v>
+      </c>
+      <c r="C58" s="7">
+        <v>830</v>
+      </c>
+      <c r="D58" s="7">
+        <v>0</v>
+      </c>
+      <c r="E58" s="7">
+        <v>5</v>
+      </c>
+      <c r="F58" s="7">
+        <v>6</v>
+      </c>
+      <c r="G58" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A59" s="7">
+        <v>2087</v>
+      </c>
+      <c r="B59" s="7">
+        <v>851</v>
+      </c>
+      <c r="C59" s="7">
+        <v>840</v>
+      </c>
+      <c r="D59" s="7">
+        <v>0</v>
+      </c>
+      <c r="E59" s="7">
+        <v>5</v>
+      </c>
+      <c r="F59" s="8">
+        <v>0</v>
+      </c>
+      <c r="G59" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A60" s="7">
+        <v>2088</v>
+      </c>
+      <c r="B60" s="7">
+        <v>861</v>
+      </c>
+      <c r="C60" s="7">
+        <v>850</v>
+      </c>
+      <c r="D60" s="7">
+        <v>0</v>
+      </c>
+      <c r="E60" s="7">
+        <v>5</v>
+      </c>
+      <c r="F60" s="8">
+        <v>0</v>
+      </c>
+      <c r="G60" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A61" s="7">
+        <v>2089</v>
+      </c>
+      <c r="B61" s="7">
+        <v>871</v>
+      </c>
+      <c r="C61" s="7">
+        <v>860</v>
+      </c>
+      <c r="D61" s="7">
+        <v>0</v>
+      </c>
+      <c r="E61" s="8">
+        <v>0</v>
+      </c>
+      <c r="F61" s="8">
+        <v>0</v>
+      </c>
+      <c r="G61" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A62" s="7">
+        <v>2090</v>
+      </c>
+      <c r="B62" s="7">
+        <v>881</v>
+      </c>
+      <c r="C62" s="7">
+        <v>870</v>
+      </c>
+      <c r="D62" s="7">
+        <v>0</v>
+      </c>
+      <c r="E62" s="8">
+        <v>0</v>
+      </c>
+      <c r="F62" s="8">
+        <v>0</v>
+      </c>
+      <c r="G62" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A63" s="7">
+        <v>2091</v>
+      </c>
+      <c r="B63" s="7">
+        <v>891</v>
+      </c>
+      <c r="C63" s="7">
+        <v>880</v>
+      </c>
+      <c r="D63" s="7">
+        <v>0</v>
+      </c>
+      <c r="E63" s="8">
+        <v>0</v>
+      </c>
+      <c r="F63" s="8">
+        <v>0</v>
+      </c>
+      <c r="G63" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A64" s="7">
+        <v>2092</v>
+      </c>
+      <c r="B64" s="7">
+        <v>901</v>
+      </c>
+      <c r="C64" s="7">
+        <v>890</v>
+      </c>
+      <c r="D64" s="7">
+        <v>0</v>
+      </c>
+      <c r="E64" s="8">
+        <v>0</v>
+      </c>
+      <c r="F64" s="8">
+        <v>0</v>
+      </c>
+      <c r="G64" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A65" s="7">
+        <v>2093</v>
+      </c>
+      <c r="B65" s="7">
+        <v>911</v>
+      </c>
+      <c r="C65" s="7">
+        <v>900</v>
+      </c>
+      <c r="D65" s="7">
+        <v>0</v>
+      </c>
+      <c r="E65" s="8">
+        <v>0</v>
+      </c>
+      <c r="F65" s="8">
+        <v>0</v>
+      </c>
+      <c r="G65" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A66" s="7">
+        <v>2094</v>
+      </c>
+      <c r="B66" s="7">
+        <v>921</v>
+      </c>
+      <c r="C66" s="7">
+        <v>910</v>
+      </c>
+      <c r="D66" s="7">
+        <v>0</v>
+      </c>
+      <c r="E66" s="8">
+        <v>0</v>
+      </c>
+      <c r="F66" s="8">
+        <v>0</v>
+      </c>
+      <c r="G66" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A67" s="7">
+        <v>2095</v>
+      </c>
+      <c r="B67" s="7">
+        <v>931</v>
+      </c>
+      <c r="C67" s="7">
+        <v>920</v>
+      </c>
+      <c r="D67" s="7">
+        <v>0</v>
+      </c>
+      <c r="E67" s="8">
+        <v>0</v>
+      </c>
+      <c r="F67" s="8">
+        <v>0</v>
+      </c>
+      <c r="G67" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A68" s="7">
+        <v>2096</v>
+      </c>
+      <c r="B68" s="7">
+        <v>941</v>
+      </c>
+      <c r="C68" s="7">
+        <v>930</v>
+      </c>
+      <c r="D68" s="7">
+        <v>0</v>
+      </c>
+      <c r="E68" s="8">
+        <v>0</v>
+      </c>
+      <c r="F68" s="8">
+        <v>0</v>
+      </c>
+      <c r="G68" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A69" s="7">
+        <v>2097</v>
+      </c>
+      <c r="B69" s="7">
+        <v>951</v>
+      </c>
+      <c r="C69" s="7">
+        <v>940</v>
+      </c>
+      <c r="D69" s="7">
+        <v>0</v>
+      </c>
+      <c r="E69" s="8">
+        <v>0</v>
+      </c>
+      <c r="F69" s="8">
+        <v>0</v>
+      </c>
+      <c r="G69" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A70" s="7">
+        <v>2098</v>
+      </c>
+      <c r="B70" s="7">
+        <v>961</v>
+      </c>
+      <c r="C70" s="7">
+        <v>950</v>
+      </c>
+      <c r="D70" s="7">
+        <v>0</v>
+      </c>
+      <c r="E70" s="8">
+        <v>0</v>
+      </c>
+      <c r="F70" s="8">
+        <v>0</v>
+      </c>
+      <c r="G70" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A71" s="7">
+        <v>2099</v>
+      </c>
+      <c r="B71" s="7">
+        <v>971</v>
+      </c>
+      <c r="C71" s="7">
+        <v>960</v>
+      </c>
+      <c r="D71" s="7">
+        <v>0</v>
+      </c>
+      <c r="E71" s="8">
+        <v>0</v>
+      </c>
+      <c r="F71" s="8">
+        <v>0</v>
+      </c>
+      <c r="G71" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A72" s="7">
+        <v>2100</v>
+      </c>
+      <c r="B72" s="7">
+        <v>981</v>
+      </c>
+      <c r="C72" s="7">
+        <v>970</v>
+      </c>
+      <c r="D72" s="7">
+        <v>0</v>
+      </c>
+      <c r="E72" s="8">
+        <v>0</v>
+      </c>
+      <c r="F72" s="8">
+        <v>0</v>
+      </c>
+      <c r="G72" s="7">
         <v>0</v>
       </c>
     </row>

</xml_diff>